<commit_message>
Scan 1 fixes: risk responds-to test with evidence quotes, naming rules, programme class and the money ladder
</commit_message>
<xml_diff>
--- a/bhutan/budget_layer_all_years.xlsx
+++ b/bhutan/budget_layer_all_years.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,6 +468,21 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>source_file</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>programme_class</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>class_source</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>strategy_name_source</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Denominator fixed: nested programme levels detected per head, readability gate, ceiling capped on programme sums
</commit_message>
<xml_diff>
--- a/bhutan/budget_layer_all_years.xlsx
+++ b/bhutan/budget_layer_all_years.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="budget_all_years" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="programs_wide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reconciliation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_quality" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="national_total" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reconciliation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_quality" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -528,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,27 +540,32 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>strategy_code</t>
+          <t>head_total</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>strategy_total</t>
+          <t>programme_total</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>program_sum</t>
+          <t>gap_pct</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>diff</t>
+          <t>basis</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>nested_heads</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>national</t>
         </is>
       </c>
     </row>
@@ -580,6 +586,52 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>fiscal_year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>strategy_code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>strategy_total</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>program_sum</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>diff</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>severity</t>
         </is>
       </c>

</xml_diff>